<commit_message>
Sprint Plan, Product Backlog Updates and Cleanup
</commit_message>
<xml_diff>
--- a/Business Analysis/checkupp_product_backlog.xlsx
+++ b/Business Analysis/checkupp_product_backlog.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ANODIAM\CheckUpp\Business Analysis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\CheckUpp\Business Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEE681DB-26F8-4DDB-97C1-DE66BE59847B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC7F28F7-BD9A-4F0F-808E-8B7A5B8CE6F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -275,14 +275,6 @@
     <t>I can access them in app</t>
   </si>
   <si>
-    <t>1. The logged-in user must be able to select one or more health documents (e.g., reports) from their local device for upload to the Document Wallet.
-2. The selected health documents must be uploaded securely to the app's cloud storage and associated with the logged-in user's account.
-3. A confirmation message must be displayed to the user after each document has been successfully uploaded.
-4. If a document upload fails, an appropriate error message must be displayed, and the user must be able to retry the upload without affecting previously uploaded documents.
-5. Document wallet must list all the uploaded documents with name and date.
-6. User must be able to interact with the options to download, view and delete options for each document stored in the Document Wallet.</t>
-  </si>
-  <si>
     <t>Slide 11</t>
   </si>
   <si>
@@ -293,16 +285,6 @@
   </si>
   <si>
     <t>delete the documents in my document wallet from the app cloud storage</t>
-  </si>
-  <si>
-    <t>1. User must be able to select the Delete option for any document stored in the Documents section of the Document Wallet.
-2. A confirmation prompt (Are you sure you want to delete this file?) must be displayed before the selected document is permanently deleted from the app's cloud storage.
-3. The selected document must be permanently removed from the logged-in user's Document Wallet and the app's cloud storage after the deletion is confirmed.
-4. The deleted document must no longer be visible or accessible in the Document Wallet after successful deletion..
-5. If the document cannot be deleted, an appropriate error message (File could not be deleted, please try again) must be displayed, and the document must remain available in the Document Wallet until the deletion is successfully completed.</t>
-  </si>
-  <si>
-    <t>view and open a document stored in my document wallet</t>
   </si>
   <si>
     <t>I can review my health records at any time</t>
@@ -340,13 +322,6 @@
   </si>
   <si>
     <t>Delete my e-script links from the app's cloud storage</t>
-  </si>
-  <si>
-    <t>1. User must be able to select the Delete option for any e-script link stored in the Links section of the Document Wallet.
-2. A confirmation prompt (e.g., "Are you sure you want to delete this link?") must be displayed before the selected e-script link is permanently deleted from the app's cloud storage.
-3. The selected e-script link must be permanently removed from the logged-in user's Document Wallet and the app's cloud storage after the deletion is confirmed.
-4. The deleted e-script link must no longer be visible or accessible in the Links section after successful deletion.
-5. If the e-script link cannot be deleted, an appropriate error message (e.g., "Link could not be deleted, please try again.") must be displayed, and the link must remain available in the Document Wallet until the deletion is successfully completed.</t>
   </si>
   <si>
     <t>Health Checks Hub</t>
@@ -5251,44 +5226,67 @@
     <t>I can save the document to my local device storage without having to open it first</t>
   </si>
   <si>
-    <t>1. User must be able to initiate a download by tapping the Download icon on the document card or within the expanded action menu.
+    <t>1. If a document cannot be opened, an appropriate error message ('Could not open file') must be displayed, and the user must be able to retry opening the document.
+2. The selected document must be displayed in a readable format using the device's supported document viewer (Drive PDF Viewer, OneDrive PDF viewer, Adobe Acrobat Reader etc).
+3. The explicit "Download" button must be removed from this view screen, as it is now an independent card action.</t>
+  </si>
+  <si>
+    <t>access document actions through an organized card layout with an overflow menu</t>
+  </si>
+  <si>
+    <t>the interface remains uncluttered and accidental deletions are prevented</t>
+  </si>
+  <si>
+    <t>access link actions through a responsive card layout</t>
+  </si>
+  <si>
+    <t>the interface remains uncluttered regardless of my device's screen size</t>
+  </si>
+  <si>
+    <t>1. The logged-in user must be able to select one or more health documents (e.g., reports) from their local device for upload to the Document Wallet.
+2. The selected health documents must be uploaded securely to the app's Firebase Storage and associated with the logged-in user's account.
+3. A confirmation message must be displayed to the user after each document has been successfully uploaded.
+4. If a document upload fails, an appropriate error message must be displayed, and the user must be able to retry the upload without affecting previously uploaded documents.
+5. Document wallet must list all the uploaded documents with name and date.
+6. User must be able to interact with the options to download, view and delete options for each document stored in the Document Wallet.</t>
+  </si>
+  <si>
+    <t>1. User must be able to select the Delete option for any document stored in the Documents section of the Document Wallet.
+2. A confirmation prompt (Are you sure you want to delete this file?) must be displayed before the selected document is permanently deleted from Firebase Storage and the database.
+3. The selected document must be permanently removed from the logged-in user's Document Wallet and Firebase Storage after the deletion is confirmed.
+4. The deleted document must no longer be visible or accessible in the Document Wallet after successful deletion.
+5. If the document cannot be deleted, an appropriate error message (File could not be deleted, please try again) must be displayed, and the document must remain available in the Document Wallet until the deletion is successfully completed.</t>
+  </si>
+  <si>
+    <t>1. User must be able to initiate a download by tapping the Download option within the expanded 3-dot (kebab) action menu.
 2. The document must securely download to the user's local device storage.
 3. A success message (e.g., "Download complete") must be displayed upon completion.
 4. If the download fails, an error message must prompt the user to try again.</t>
   </si>
   <si>
-    <t>1. If a document cannot be opened, an appropriate error message ('Could not open file') must be displayed, and the user must be able to retry opening the document.
-2. The selected document must be displayed in a readable format using the device's supported document viewer (Drive PDF Viewer, OneDrive PDF viewer, Adobe Acrobat Reader etc).
-3. The explicit "Download" button must be removed from this view screen, as it is now an independent card action.</t>
-  </si>
-  <si>
-    <t>access document actions through an organized card layout with an overflow menu</t>
-  </si>
-  <si>
-    <t>the interface remains uncluttered and accidental deletions are prevented</t>
-  </si>
-  <si>
-    <t>1. If screen real estate permits, the card must display standalone icons for "Share" and "Download", plus a vertical three-dot (kebab) menu.
-2. Expanding the kebab menu must reveal the "View" and "Delete" options.
-3. Edge Case: If device screen size restricts showing two standalone icons, the card must default to showing only the "Share" icon and the kebab menu. Expanding the menu must then show "View", "Download", and "Delete".</t>
+    <t>view (open inside app) a document stored in my document wallet</t>
+  </si>
+  <si>
+    <t>1. To prevent UI clutter on small devices, the card must display a standalone icon for "Share" alongside a vertical three-dot (kebab) menu.
+2. Expanding the kebab menu must reveal the "View", "Download", and "Delete" options.</t>
   </si>
   <si>
     <t>1. User must be able to add an e-script link along with the associated text description of their choice in the Links section of the Document Wallet.
-2. All saved e-script links and their associated descriptions must be displayed as a list in the Links section of the Document Wallet.
+2. All saved e-script links and their associated descriptions must be securely saved in the database and displayed as a list in the Links section.
 3. If an e-script link cannot be saved, an appropriate error message (Link could not be saved, Try again) must be displayed, and the user must be able to retry the action without affecting previously saved links.
-4. Document wallet must list all the saved links with name and date
+4. Document wallet must list all the saved links with name and date.
 5. User must be able to interact with standalone or menu-grouped options to open, share, and delete each link.</t>
   </si>
   <si>
-    <t>access link actions through a responsive card layout</t>
-  </si>
-  <si>
-    <t>the interface remains uncluttered regardless of my device's screen size</t>
-  </si>
-  <si>
-    <t>1. If screen real estate permits, the link card must display standalone options for "Share", "Open", and "Delete".
-2. Edge Case: If the device screen size restricts showing all three options natively, the card must display the "Share" icon alongside a Hamburger Menu (three vertically stacked dots).
-3. Expanding the Hamburger Menu must reveal the "Open" and "Delete" options.</t>
+    <t>1. User must be able to select the Delete option for any e-script link stored in the Links section of the Document Wallet.
+2. A confirmation prompt (e.g., "Are you sure you want to delete this link?") must be displayed before the selected e-script link is permanently deleted from the database.
+3. The selected e-script link must be permanently removed from the logged-in user's Document Wallet and the database after the deletion is confirmed.
+4. The deleted e-script link must no longer be visible or accessible in the Links section after successful deletion.
+5. If the e-script link cannot be deleted, an appropriate error message (e.g., "Link could not be deleted, please try again.") must be displayed, and the link must remain available in the Document Wallet until the deletion is successfully completed.</t>
+  </si>
+  <si>
+    <t>1. The link card must display the "Share" icon alongside a vertical three-dot (kebab) menu to maintain consistency with the Documents tab.
+2. Expanding the kebab menu must reveal the "Open" and "Delete" options.</t>
   </si>
 </sst>
 </file>
@@ -5788,6 +5786,72 @@
     <xf numFmtId="0" fontId="2" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -5809,9 +5873,6 @@
     <xf numFmtId="0" fontId="15" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -5825,69 +5886,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6135,8 +6133,8 @@
       <c r="D1" s="71" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="65"/>
-      <c r="F1" s="65"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
       <c r="G1" s="75" t="s">
         <v>4</v>
       </c>
@@ -6148,9 +6146,9 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="65"/>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
+      <c r="A2" s="64"/>
+      <c r="B2" s="64"/>
+      <c r="C2" s="64"/>
       <c r="D2" s="4" t="s">
         <v>7</v>
       </c>
@@ -6161,8 +6159,8 @@
         <v>9</v>
       </c>
       <c r="G2" s="75"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
+      <c r="H2" s="64"/>
+      <c r="I2" s="64"/>
     </row>
     <row r="3" spans="1:9" s="5" customFormat="1" ht="108" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="76">
@@ -6175,16 +6173,16 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="E3" s="16" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="G3" s="17" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="H3" s="16" t="s">
         <v>11</v>
@@ -6200,16 +6198,16 @@
         <v>1.2</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="H4" s="16"/>
       <c r="I4" s="16"/>
@@ -6221,16 +6219,16 @@
         <v>1.3</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="H5" s="16"/>
       <c r="I5" s="16"/>
@@ -6242,16 +6240,16 @@
         <v>1.4</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="H6" s="16"/>
       <c r="I6" s="16"/>
@@ -6263,16 +6261,16 @@
         <v>1.5</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="H7" s="16"/>
       <c r="I7" s="16"/>
@@ -6284,16 +6282,16 @@
         <v>1.6</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="H8" s="16"/>
       <c r="I8" s="16"/>
@@ -6305,16 +6303,16 @@
         <v>1.7</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="G9" s="17" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="H9" s="16"/>
       <c r="I9" s="16"/>
@@ -6326,16 +6324,16 @@
         <v>1.8</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="H10" s="16"/>
       <c r="I10" s="51"/>
@@ -6418,16 +6416,16 @@
         <v>5.4</v>
       </c>
       <c r="D14" s="21" t="s">
+        <v>142</v>
+      </c>
+      <c r="E14" s="21" t="s">
+        <v>145</v>
+      </c>
+      <c r="F14" s="21" t="s">
+        <v>144</v>
+      </c>
+      <c r="G14" s="22" t="s">
         <v>146</v>
-      </c>
-      <c r="E14" s="21" t="s">
-        <v>149</v>
-      </c>
-      <c r="F14" s="21" t="s">
-        <v>148</v>
-      </c>
-      <c r="G14" s="22" t="s">
-        <v>150</v>
       </c>
       <c r="H14" s="23"/>
       <c r="I14" s="21"/>
@@ -6439,52 +6437,52 @@
         <v>5.5</v>
       </c>
       <c r="D15" s="21" t="s">
+        <v>139</v>
+      </c>
+      <c r="E15" s="21" t="s">
         <v>143</v>
       </c>
-      <c r="E15" s="21" t="s">
-        <v>147</v>
-      </c>
       <c r="F15" s="21" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="G15" s="22" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="H15" s="23"/>
       <c r="I15" s="21"/>
     </row>
     <row r="16" spans="1:9" s="14" customFormat="1" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="80">
+      <c r="A16" s="58">
         <v>6</v>
       </c>
-      <c r="B16" s="80" t="s">
+      <c r="B16" s="58" t="s">
         <v>25</v>
       </c>
-      <c r="C16" s="21">
+      <c r="C16" s="24">
         <v>6.1</v>
       </c>
-      <c r="D16" s="21" t="s">
+      <c r="D16" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="E16" s="21" t="s">
+      <c r="E16" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="F16" s="21" t="s">
+      <c r="F16" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="G16" s="22" t="s">
+      <c r="G16" s="25" t="s">
+        <v>324</v>
+      </c>
+      <c r="H16" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="H16" s="23" t="s">
+      <c r="I16" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="I16" s="21" t="s">
-        <v>31</v>
-      </c>
     </row>
     <row r="17" spans="1:9" s="6" customFormat="1" ht="144" x14ac:dyDescent="0.3">
-      <c r="A17" s="81"/>
-      <c r="B17" s="81"/>
+      <c r="A17" s="59"/>
+      <c r="B17" s="59"/>
       <c r="C17" s="24">
         <v>6.2</v>
       </c>
@@ -6492,20 +6490,20 @@
         <v>26</v>
       </c>
       <c r="E17" s="24" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="F17" s="24" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="G17" s="25" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="H17" s="26"/>
       <c r="I17" s="24"/>
     </row>
     <row r="18" spans="1:9" s="6" customFormat="1" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="81"/>
-      <c r="B18" s="81"/>
+      <c r="A18" s="59"/>
+      <c r="B18" s="59"/>
       <c r="C18" s="24">
         <v>6.3</v>
       </c>
@@ -6513,20 +6511,20 @@
         <v>26</v>
       </c>
       <c r="E18" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="F18" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="F18" s="24" t="s">
-        <v>33</v>
-      </c>
       <c r="G18" s="25" t="s">
-        <v>34</v>
+        <v>325</v>
       </c>
       <c r="H18" s="26"/>
       <c r="I18" s="24"/>
     </row>
     <row r="19" spans="1:9" s="6" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A19" s="81"/>
-      <c r="B19" s="81"/>
+      <c r="A19" s="59"/>
+      <c r="B19" s="59"/>
       <c r="C19" s="27">
         <v>6.4</v>
       </c>
@@ -6534,24 +6532,24 @@
         <v>26</v>
       </c>
       <c r="E19" s="24" t="s">
-        <v>35</v>
+        <v>327</v>
       </c>
       <c r="F19" s="24" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G19" s="25" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="H19" s="26" t="s">
+        <v>29</v>
+      </c>
+      <c r="I19" s="24" t="s">
         <v>30</v>
-      </c>
-      <c r="I19" s="24" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="20" spans="1:9" s="6" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A20" s="52"/>
-      <c r="B20" s="81"/>
+      <c r="B20" s="59"/>
       <c r="C20" s="24">
         <v>6.5</v>
       </c>
@@ -6559,20 +6557,20 @@
         <v>26</v>
       </c>
       <c r="E20" s="24" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="F20" s="24" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="G20" s="25" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="H20" s="26"/>
       <c r="I20" s="24"/>
     </row>
-    <row r="21" spans="1:9" s="6" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" s="6" customFormat="1" ht="72" x14ac:dyDescent="0.3">
       <c r="A21" s="52"/>
-      <c r="B21" s="82"/>
+      <c r="B21" s="70"/>
       <c r="C21" s="24">
         <v>6.6</v>
       </c>
@@ -6580,125 +6578,125 @@
         <v>26</v>
       </c>
       <c r="E21" s="24" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="F21" s="24" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="G21" s="25" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="H21" s="26"/>
       <c r="I21" s="24"/>
     </row>
     <row r="22" spans="1:9" s="6" customFormat="1" ht="144" x14ac:dyDescent="0.3">
-      <c r="A22" s="83">
+      <c r="A22" s="60">
         <v>7</v>
       </c>
-      <c r="B22" s="80" t="s">
-        <v>37</v>
+      <c r="B22" s="58" t="s">
+        <v>34</v>
       </c>
       <c r="C22" s="24">
         <v>7.1</v>
       </c>
       <c r="D22" s="24" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E22" s="24" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F22" s="24" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="G22" s="25" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="H22" s="26" t="s">
+        <v>29</v>
+      </c>
+      <c r="I22" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="I22" s="24" t="s">
-        <v>31</v>
-      </c>
     </row>
     <row r="23" spans="1:9" s="6" customFormat="1" ht="72" x14ac:dyDescent="0.3">
-      <c r="A23" s="84"/>
-      <c r="B23" s="81"/>
+      <c r="A23" s="61"/>
+      <c r="B23" s="59"/>
       <c r="C23" s="24">
         <v>7.2</v>
       </c>
       <c r="D23" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="E23" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="E23" s="24" t="s">
-        <v>41</v>
-      </c>
       <c r="F23" s="24" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G23" s="25" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="H23" s="26"/>
       <c r="I23" s="24" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="24" spans="1:9" s="6" customFormat="1" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="A24" s="84"/>
-      <c r="B24" s="81"/>
+      <c r="A24" s="61"/>
+      <c r="B24" s="59"/>
       <c r="C24" s="24">
         <v>7.3</v>
       </c>
       <c r="D24" s="24" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E24" s="24" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="F24" s="24" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="G24" s="25" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="H24" s="26"/>
       <c r="I24" s="24"/>
     </row>
-    <row r="25" spans="1:9" s="6" customFormat="1" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A25" s="85"/>
-      <c r="B25" s="81"/>
+    <row r="25" spans="1:9" s="6" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="A25" s="62"/>
+      <c r="B25" s="59"/>
       <c r="C25" s="24">
         <v>7.4</v>
       </c>
       <c r="D25" s="24" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E25" s="24" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="F25" s="24" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G25" s="25" t="s">
-        <v>47</v>
+        <v>330</v>
       </c>
       <c r="H25" s="26"/>
       <c r="I25" s="24"/>
     </row>
-    <row r="26" spans="1:9" s="6" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" s="6" customFormat="1" ht="72" x14ac:dyDescent="0.3">
       <c r="A26" s="52"/>
-      <c r="B26" s="82"/>
+      <c r="B26" s="70"/>
       <c r="C26" s="24">
         <v>7.5</v>
       </c>
       <c r="D26" s="24" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E26" s="24" t="s">
-        <v>329</v>
+        <v>322</v>
       </c>
       <c r="F26" s="24" t="s">
-        <v>330</v>
+        <v>323</v>
       </c>
       <c r="G26" s="25" t="s">
         <v>331</v>
@@ -6707,1075 +6705,1075 @@
       <c r="I26" s="24"/>
     </row>
     <row r="27" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A27" s="89">
+      <c r="A27" s="67">
         <v>8</v>
       </c>
-      <c r="B27" s="89" t="s">
-        <v>48</v>
+      <c r="B27" s="67" t="s">
+        <v>44</v>
       </c>
       <c r="C27" s="28">
         <v>9.1999999999999993</v>
       </c>
       <c r="D27" s="28" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E27" s="28" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="F27" s="28" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G27" s="29" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="H27" s="28"/>
       <c r="I27" s="28" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="28" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A28" s="90"/>
-      <c r="B28" s="90"/>
+      <c r="A28" s="68"/>
+      <c r="B28" s="68"/>
       <c r="C28" s="28">
         <v>9.3000000000000007</v>
       </c>
       <c r="D28" s="28" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E28" s="28" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="F28" s="28" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="G28" s="29" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="H28" s="28"/>
       <c r="I28" s="28" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="29" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A29" s="91"/>
-      <c r="B29" s="91"/>
+      <c r="A29" s="69"/>
+      <c r="B29" s="69"/>
       <c r="C29" s="28">
         <v>9.4</v>
       </c>
       <c r="D29" s="28" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E29" s="28" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="F29" s="28" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G29" s="29" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="H29" s="28"/>
       <c r="I29" s="28" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="30" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="87">
+      <c r="A30" s="65">
         <v>12</v>
       </c>
-      <c r="B30" s="87" t="s">
-        <v>58</v>
+      <c r="B30" s="65" t="s">
+        <v>54</v>
       </c>
       <c r="C30" s="30">
         <v>12.1</v>
       </c>
       <c r="D30" s="30" t="s">
+        <v>55</v>
+      </c>
+      <c r="E30" s="30" t="s">
+        <v>56</v>
+      </c>
+      <c r="F30" s="30" t="s">
+        <v>57</v>
+      </c>
+      <c r="G30" s="31" t="s">
+        <v>58</v>
+      </c>
+      <c r="H30" s="30" t="s">
         <v>59</v>
       </c>
-      <c r="E30" s="30" t="s">
+      <c r="I30" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="F30" s="30" t="s">
-        <v>61</v>
-      </c>
-      <c r="G30" s="31" t="s">
-        <v>62</v>
-      </c>
-      <c r="H30" s="30" t="s">
-        <v>63</v>
-      </c>
-      <c r="I30" s="30" t="s">
-        <v>64</v>
-      </c>
     </row>
     <row r="31" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A31" s="87"/>
-      <c r="B31" s="87"/>
+      <c r="A31" s="65"/>
+      <c r="B31" s="65"/>
       <c r="C31" s="30">
         <v>12.2</v>
       </c>
       <c r="D31" s="30" t="s">
+        <v>55</v>
+      </c>
+      <c r="E31" s="30" t="s">
+        <v>61</v>
+      </c>
+      <c r="F31" s="30" t="s">
+        <v>62</v>
+      </c>
+      <c r="G31" s="31" t="s">
+        <v>63</v>
+      </c>
+      <c r="H31" s="30" t="s">
         <v>59</v>
       </c>
-      <c r="E31" s="30" t="s">
-        <v>65</v>
-      </c>
-      <c r="F31" s="30" t="s">
-        <v>66</v>
-      </c>
-      <c r="G31" s="31" t="s">
-        <v>67</v>
-      </c>
-      <c r="H31" s="30" t="s">
-        <v>63</v>
-      </c>
       <c r="I31" s="30" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="32" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="87"/>
-      <c r="B32" s="87"/>
+      <c r="A32" s="65"/>
+      <c r="B32" s="65"/>
       <c r="C32" s="30">
         <v>12.3</v>
       </c>
       <c r="D32" s="30" t="s">
+        <v>55</v>
+      </c>
+      <c r="E32" s="30" t="s">
+        <v>64</v>
+      </c>
+      <c r="F32" s="30" t="s">
+        <v>65</v>
+      </c>
+      <c r="G32" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="H32" s="30" t="s">
         <v>59</v>
       </c>
-      <c r="E32" s="30" t="s">
-        <v>68</v>
-      </c>
-      <c r="F32" s="30" t="s">
-        <v>69</v>
-      </c>
-      <c r="G32" s="31" t="s">
-        <v>70</v>
-      </c>
-      <c r="H32" s="30" t="s">
-        <v>63</v>
-      </c>
       <c r="I32" s="30" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="33" spans="1:9" s="6" customFormat="1" ht="123.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="87"/>
-      <c r="B33" s="87"/>
+      <c r="A33" s="65"/>
+      <c r="B33" s="65"/>
       <c r="C33" s="30">
         <v>12.4</v>
       </c>
       <c r="D33" s="30" t="s">
+        <v>55</v>
+      </c>
+      <c r="E33" s="30" t="s">
+        <v>220</v>
+      </c>
+      <c r="F33" s="30" t="s">
+        <v>221</v>
+      </c>
+      <c r="G33" s="31" t="s">
+        <v>222</v>
+      </c>
+      <c r="H33" s="30" t="s">
         <v>59</v>
       </c>
-      <c r="E33" s="30" t="s">
-        <v>224</v>
-      </c>
-      <c r="F33" s="30" t="s">
-        <v>225</v>
-      </c>
-      <c r="G33" s="31" t="s">
-        <v>226</v>
-      </c>
-      <c r="H33" s="30" t="s">
-        <v>63</v>
-      </c>
       <c r="I33" s="30" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="34" spans="1:9" s="6" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A34" s="87"/>
-      <c r="B34" s="87"/>
+      <c r="A34" s="65"/>
+      <c r="B34" s="65"/>
       <c r="C34" s="30">
         <v>12.5</v>
       </c>
       <c r="D34" s="30" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="E34" s="30" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="F34" s="30" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="G34" s="31" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H34" s="30" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="I34" s="30" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="35" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A35" s="88">
+      <c r="A35" s="66">
         <v>14</v>
       </c>
-      <c r="B35" s="88" t="s">
-        <v>74</v>
+      <c r="B35" s="66" t="s">
+        <v>70</v>
       </c>
       <c r="C35" s="34">
         <v>14.1</v>
       </c>
       <c r="D35" s="35" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E35" s="35" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="F35" s="35" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="G35" s="36" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="H35" s="34" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="I35" s="34" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="36" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A36" s="88"/>
-      <c r="B36" s="88"/>
+      <c r="A36" s="66"/>
+      <c r="B36" s="66"/>
       <c r="C36" s="34">
         <v>14.2</v>
       </c>
       <c r="D36" s="35" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E36" s="35" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="F36" s="35" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="G36" s="36" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="H36" s="34" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="I36" s="34" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="37" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A37" s="88"/>
-      <c r="B37" s="88"/>
+      <c r="A37" s="66"/>
+      <c r="B37" s="66"/>
       <c r="C37" s="34">
         <v>14.3</v>
       </c>
       <c r="D37" s="35" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="E37" s="35" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="F37" s="35" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="G37" s="36" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="H37" s="34" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="I37" s="34" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="38" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A38" s="88"/>
-      <c r="B38" s="88"/>
+      <c r="A38" s="66"/>
+      <c r="B38" s="66"/>
       <c r="C38" s="34">
         <v>14.4</v>
       </c>
       <c r="D38" s="35" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E38" s="35" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="F38" s="35" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="G38" s="36" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="H38" s="34" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="I38" s="34" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="39" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A39" s="88"/>
-      <c r="B39" s="88"/>
+      <c r="A39" s="66"/>
+      <c r="B39" s="66"/>
       <c r="C39" s="34">
         <v>14.5</v>
       </c>
       <c r="D39" s="35" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E39" s="35" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="F39" s="35" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="G39" s="36" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="H39" s="34" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="I39" s="34" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="40" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A40" s="88"/>
-      <c r="B40" s="88"/>
+      <c r="A40" s="66"/>
+      <c r="B40" s="66"/>
       <c r="C40" s="34">
         <v>14.6</v>
       </c>
       <c r="D40" s="35" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E40" s="35" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="F40" s="35" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="G40" s="36" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="H40" s="34" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="I40" s="34" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="41" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A41" s="88"/>
-      <c r="B41" s="88"/>
+      <c r="A41" s="66"/>
+      <c r="B41" s="66"/>
       <c r="C41" s="34">
         <v>14.7</v>
       </c>
       <c r="D41" s="35" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E41" s="35" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="F41" s="35" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="G41" s="36" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="H41" s="34" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="I41" s="34" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="42" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A42" s="88"/>
-      <c r="B42" s="88"/>
+      <c r="A42" s="66"/>
+      <c r="B42" s="66"/>
       <c r="C42" s="34">
         <v>14.8</v>
       </c>
       <c r="D42" s="35" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E42" s="35" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="F42" s="35" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="G42" s="36" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="H42" s="34" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="I42" s="34" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="43" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A43" s="88"/>
-      <c r="B43" s="88"/>
+      <c r="A43" s="66"/>
+      <c r="B43" s="66"/>
       <c r="C43" s="34">
         <v>14.9</v>
       </c>
       <c r="D43" s="35" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E43" s="35" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="F43" s="35" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="G43" s="36" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="H43" s="34" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="I43" s="34" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="44" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A44" s="88"/>
-      <c r="B44" s="88"/>
+      <c r="A44" s="66"/>
+      <c r="B44" s="66"/>
       <c r="C44" s="34">
         <v>14.1</v>
       </c>
       <c r="D44" s="35" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E44" s="35" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="F44" s="35" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="G44" s="36" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="H44" s="34" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="I44" s="34" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="45" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A45" s="88"/>
-      <c r="B45" s="88"/>
+      <c r="A45" s="66"/>
+      <c r="B45" s="66"/>
       <c r="C45" s="34">
         <v>14.11</v>
       </c>
       <c r="D45" s="35" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E45" s="35" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="F45" s="35" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="G45" s="36" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="H45" s="34" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="I45" s="34" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="46" spans="1:9" s="6" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A46" s="86">
+      <c r="A46" s="63">
         <v>15</v>
       </c>
-      <c r="B46" s="86" t="s">
-        <v>78</v>
+      <c r="B46" s="63" t="s">
+        <v>74</v>
       </c>
       <c r="C46" s="37">
         <v>15.1</v>
       </c>
       <c r="D46" s="37" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E46" s="37" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F46" s="37" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="G46" s="38" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="H46" s="37" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="I46" s="37" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="47" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A47" s="65"/>
-      <c r="B47" s="65"/>
+      <c r="A47" s="64"/>
+      <c r="B47" s="64"/>
       <c r="C47" s="37">
         <v>15.2</v>
       </c>
       <c r="D47" s="37" t="s">
+        <v>75</v>
+      </c>
+      <c r="E47" s="37" t="s">
+        <v>78</v>
+      </c>
+      <c r="F47" s="37" t="s">
         <v>79</v>
       </c>
-      <c r="E47" s="37" t="s">
-        <v>82</v>
-      </c>
-      <c r="F47" s="37" t="s">
-        <v>83</v>
-      </c>
       <c r="G47" s="38" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="H47" s="37" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="I47" s="37" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="48" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A48" s="65"/>
-      <c r="B48" s="65"/>
+      <c r="A48" s="64"/>
+      <c r="B48" s="64"/>
       <c r="C48" s="37">
         <v>15.3</v>
       </c>
       <c r="D48" s="37" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E48" s="37" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F48" s="37" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="G48" s="38" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="H48" s="37" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="I48" s="37" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="49" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A49" s="65"/>
-      <c r="B49" s="65"/>
+      <c r="A49" s="64"/>
+      <c r="B49" s="64"/>
       <c r="C49" s="37">
         <v>15.4</v>
       </c>
       <c r="D49" s="37" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E49" s="37" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="F49" s="37" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="G49" s="38" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="H49" s="37" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="I49" s="37" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="50" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A50" s="65"/>
-      <c r="B50" s="65"/>
+      <c r="A50" s="64"/>
+      <c r="B50" s="64"/>
       <c r="C50" s="37">
         <v>15.5</v>
       </c>
       <c r="D50" s="37" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E50" s="37" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="F50" s="37" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="G50" s="38" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="H50" s="37" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="I50" s="37" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="51" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A51" s="65"/>
-      <c r="B51" s="65"/>
+      <c r="A51" s="64"/>
+      <c r="B51" s="64"/>
       <c r="C51" s="37">
         <v>15.6</v>
       </c>
       <c r="D51" s="37" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E51" s="37" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F51" s="37" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="G51" s="38" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="H51" s="37" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="I51" s="37" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="52" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A52" s="65"/>
-      <c r="B52" s="65"/>
+      <c r="A52" s="64"/>
+      <c r="B52" s="64"/>
       <c r="C52" s="37">
         <v>15.7</v>
       </c>
       <c r="D52" s="37" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E52" s="37" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="F52" s="37" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="G52" s="38" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="H52" s="37" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="I52" s="37" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="53" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A53" s="65"/>
-      <c r="B53" s="65"/>
+      <c r="A53" s="64"/>
+      <c r="B53" s="64"/>
       <c r="C53" s="37">
         <v>15.8</v>
       </c>
       <c r="D53" s="37" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E53" s="37" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F53" s="37" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="G53" s="38" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="H53" s="37" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="I53" s="37" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="54" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A54" s="64">
+      <c r="A54" s="86">
         <v>16</v>
       </c>
-      <c r="B54" s="64" t="s">
-        <v>93</v>
+      <c r="B54" s="86" t="s">
+        <v>89</v>
       </c>
       <c r="C54" s="39">
         <v>16.100000000000001</v>
       </c>
       <c r="D54" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="E54" s="40" t="s">
+        <v>91</v>
+      </c>
+      <c r="F54" s="40" t="s">
+        <v>92</v>
+      </c>
+      <c r="G54" s="41" t="s">
+        <v>155</v>
+      </c>
+      <c r="H54" s="40" t="s">
+        <v>93</v>
+      </c>
+      <c r="I54" s="40" t="s">
         <v>94</v>
       </c>
-      <c r="E54" s="40" t="s">
-        <v>95</v>
-      </c>
-      <c r="F54" s="40" t="s">
-        <v>96</v>
-      </c>
-      <c r="G54" s="41" t="s">
-        <v>159</v>
-      </c>
-      <c r="H54" s="40" t="s">
-        <v>97</v>
-      </c>
-      <c r="I54" s="40" t="s">
-        <v>98</v>
-      </c>
     </row>
     <row r="55" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A55" s="64"/>
-      <c r="B55" s="64"/>
+      <c r="A55" s="86"/>
+      <c r="B55" s="86"/>
       <c r="C55" s="39">
         <v>16.2</v>
       </c>
       <c r="D55" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="E55" s="40" t="s">
+        <v>95</v>
+      </c>
+      <c r="F55" s="40" t="s">
+        <v>96</v>
+      </c>
+      <c r="G55" s="41" t="s">
+        <v>156</v>
+      </c>
+      <c r="H55" s="40" t="s">
+        <v>93</v>
+      </c>
+      <c r="I55" s="40" t="s">
         <v>94</v>
       </c>
-      <c r="E55" s="40" t="s">
-        <v>99</v>
-      </c>
-      <c r="F55" s="40" t="s">
-        <v>100</v>
-      </c>
-      <c r="G55" s="41" t="s">
-        <v>160</v>
-      </c>
-      <c r="H55" s="40" t="s">
-        <v>97</v>
-      </c>
-      <c r="I55" s="40" t="s">
-        <v>98</v>
-      </c>
     </row>
     <row r="56" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A56" s="64"/>
-      <c r="B56" s="64"/>
+      <c r="A56" s="86"/>
+      <c r="B56" s="86"/>
       <c r="C56" s="39">
         <v>16.3</v>
       </c>
       <c r="D56" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="E56" s="40" t="s">
+        <v>97</v>
+      </c>
+      <c r="F56" s="40" t="s">
+        <v>98</v>
+      </c>
+      <c r="G56" s="41" t="s">
+        <v>157</v>
+      </c>
+      <c r="H56" s="40" t="s">
+        <v>93</v>
+      </c>
+      <c r="I56" s="40" t="s">
         <v>94</v>
       </c>
-      <c r="E56" s="40" t="s">
-        <v>101</v>
-      </c>
-      <c r="F56" s="40" t="s">
-        <v>102</v>
-      </c>
-      <c r="G56" s="41" t="s">
-        <v>161</v>
-      </c>
-      <c r="H56" s="40" t="s">
-        <v>97</v>
-      </c>
-      <c r="I56" s="40" t="s">
-        <v>98</v>
-      </c>
     </row>
     <row r="57" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A57" s="64"/>
-      <c r="B57" s="64"/>
+      <c r="A57" s="86"/>
+      <c r="B57" s="86"/>
       <c r="C57" s="39">
         <v>16.399999999999999</v>
       </c>
       <c r="D57" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="E57" s="40" t="s">
+        <v>99</v>
+      </c>
+      <c r="F57" s="40" t="s">
+        <v>100</v>
+      </c>
+      <c r="G57" s="41" t="s">
+        <v>158</v>
+      </c>
+      <c r="H57" s="40" t="s">
+        <v>93</v>
+      </c>
+      <c r="I57" s="40" t="s">
         <v>94</v>
       </c>
-      <c r="E57" s="40" t="s">
-        <v>103</v>
-      </c>
-      <c r="F57" s="40" t="s">
-        <v>104</v>
-      </c>
-      <c r="G57" s="41" t="s">
-        <v>162</v>
-      </c>
-      <c r="H57" s="40" t="s">
-        <v>97</v>
-      </c>
-      <c r="I57" s="40" t="s">
-        <v>98</v>
-      </c>
     </row>
     <row r="58" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A58" s="64"/>
-      <c r="B58" s="64"/>
+      <c r="A58" s="86"/>
+      <c r="B58" s="86"/>
       <c r="C58" s="39">
         <v>16.5</v>
       </c>
       <c r="D58" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="E58" s="40" t="s">
+        <v>101</v>
+      </c>
+      <c r="F58" s="40" t="s">
+        <v>102</v>
+      </c>
+      <c r="G58" s="41" t="s">
+        <v>159</v>
+      </c>
+      <c r="H58" s="40" t="s">
+        <v>93</v>
+      </c>
+      <c r="I58" s="40" t="s">
         <v>94</v>
       </c>
-      <c r="E58" s="40" t="s">
-        <v>105</v>
-      </c>
-      <c r="F58" s="40" t="s">
-        <v>106</v>
-      </c>
-      <c r="G58" s="41" t="s">
-        <v>163</v>
-      </c>
-      <c r="H58" s="40" t="s">
-        <v>97</v>
-      </c>
-      <c r="I58" s="40" t="s">
-        <v>98</v>
-      </c>
     </row>
     <row r="59" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A59" s="65"/>
-      <c r="B59" s="65"/>
+      <c r="A59" s="64"/>
+      <c r="B59" s="64"/>
       <c r="C59" s="39">
         <v>16.600000000000001</v>
       </c>
       <c r="D59" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="E59" s="40" t="s">
+        <v>103</v>
+      </c>
+      <c r="F59" s="40" t="s">
+        <v>104</v>
+      </c>
+      <c r="G59" s="41" t="s">
+        <v>160</v>
+      </c>
+      <c r="H59" s="40" t="s">
+        <v>93</v>
+      </c>
+      <c r="I59" s="40" t="s">
         <v>94</v>
       </c>
-      <c r="E59" s="40" t="s">
-        <v>107</v>
-      </c>
-      <c r="F59" s="40" t="s">
-        <v>108</v>
-      </c>
-      <c r="G59" s="41" t="s">
-        <v>164</v>
-      </c>
-      <c r="H59" s="40" t="s">
-        <v>97</v>
-      </c>
-      <c r="I59" s="40" t="s">
-        <v>98</v>
-      </c>
     </row>
     <row r="60" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A60" s="66">
+      <c r="A60" s="87">
         <v>17</v>
       </c>
-      <c r="B60" s="69" t="s">
-        <v>109</v>
+      <c r="B60" s="90" t="s">
+        <v>105</v>
       </c>
       <c r="C60" s="42">
         <v>17.100000000000001</v>
       </c>
       <c r="D60" s="42" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="E60" s="42" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="F60" s="42" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G60" s="43" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="H60" s="42" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="I60" s="42" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="61" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A61" s="67"/>
-      <c r="B61" s="69"/>
+      <c r="A61" s="88"/>
+      <c r="B61" s="90"/>
       <c r="C61" s="42">
         <v>17.2</v>
       </c>
       <c r="D61" s="42" t="s">
+        <v>106</v>
+      </c>
+      <c r="E61" s="42" t="s">
         <v>110</v>
       </c>
-      <c r="E61" s="42" t="s">
-        <v>114</v>
-      </c>
       <c r="F61" s="42" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="G61" s="43" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="H61" s="42" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="I61" s="42" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="62" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A62" s="67"/>
-      <c r="B62" s="69"/>
+      <c r="A62" s="88"/>
+      <c r="B62" s="90"/>
       <c r="C62" s="42">
         <v>17.3</v>
       </c>
       <c r="D62" s="42" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="E62" s="42" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="F62" s="42" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G62" s="43" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="H62" s="42" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="I62" s="42" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="63" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A63" s="67"/>
-      <c r="B63" s="69"/>
+      <c r="A63" s="88"/>
+      <c r="B63" s="90"/>
       <c r="C63" s="42">
         <v>17.399999999999999</v>
       </c>
       <c r="D63" s="42" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="E63" s="42" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="F63" s="42" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="G63" s="43" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="H63" s="42" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="I63" s="42" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="64" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A64" s="68"/>
-      <c r="B64" s="69"/>
+      <c r="A64" s="89"/>
+      <c r="B64" s="90"/>
       <c r="C64" s="42">
         <v>17.5</v>
       </c>
       <c r="D64" s="42" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="E64" s="42" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="F64" s="42" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="G64" s="43" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="H64" s="42" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="I64" s="42" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="65" spans="1:12" s="6" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A65" s="70">
+      <c r="A65" s="91">
         <v>18</v>
       </c>
       <c r="B65" s="72" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="C65" s="18">
         <v>18.100000000000001</v>
       </c>
       <c r="D65" s="18" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E65" s="18" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="F65" s="18" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="G65" s="19" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="H65" s="18" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="I65" s="18" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
     </row>
     <row r="66" spans="1:12" s="6" customFormat="1" ht="250.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="65"/>
+      <c r="A66" s="64"/>
       <c r="B66" s="73"/>
       <c r="C66" s="18">
         <v>18.2</v>
       </c>
       <c r="D66" s="18" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E66" s="18" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="F66" s="18" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="G66" s="19" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="H66" s="18" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="I66" s="18" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
     </row>
     <row r="67" spans="1:12" s="6" customFormat="1" ht="167.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="65"/>
+      <c r="A67" s="64"/>
       <c r="B67" s="73"/>
       <c r="C67" s="18">
         <v>18.3</v>
       </c>
       <c r="D67" s="18" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E67" s="18" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="F67" s="18" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="G67" s="19" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="H67" s="18" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="I67" s="18" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
     </row>
     <row r="68" spans="1:12" s="6" customFormat="1" ht="244.8" x14ac:dyDescent="0.3">
-      <c r="A68" s="65"/>
+      <c r="A68" s="64"/>
       <c r="B68" s="73"/>
       <c r="C68" s="18">
         <v>18.399999999999999</v>
       </c>
       <c r="D68" s="18" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E68" s="18" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="F68" s="18" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G68" s="19" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="H68" s="18" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="I68" s="18" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
     </row>
     <row r="69" spans="1:12" s="6" customFormat="1" ht="216" customHeight="1" x14ac:dyDescent="0.3">
@@ -7785,131 +7783,131 @@
         <v>18.5</v>
       </c>
       <c r="D69" s="18" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E69" s="18" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="F69" s="18" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="G69" s="19" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="H69" s="18"/>
       <c r="I69" s="18"/>
     </row>
     <row r="70" spans="1:12" s="6" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A70" s="58">
+      <c r="A70" s="80">
         <v>19</v>
       </c>
-      <c r="B70" s="61" t="s">
-        <v>124</v>
+      <c r="B70" s="83" t="s">
+        <v>120</v>
       </c>
       <c r="C70" s="44">
         <v>19.100000000000001</v>
       </c>
       <c r="D70" s="45" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="E70" s="45" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="F70" s="45" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="G70" s="46" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="H70" s="44"/>
       <c r="I70" s="47"/>
     </row>
     <row r="71" spans="1:12" s="6" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A71" s="59"/>
-      <c r="B71" s="62"/>
+      <c r="A71" s="81"/>
+      <c r="B71" s="84"/>
       <c r="C71" s="15">
         <v>19.2</v>
       </c>
       <c r="D71" s="45" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E71" s="45" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="F71" s="45" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="G71" s="46" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="H71" s="44"/>
       <c r="I71" s="47"/>
     </row>
     <row r="72" spans="1:12" s="6" customFormat="1" ht="355.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="60"/>
-      <c r="B72" s="63"/>
+      <c r="A72" s="82"/>
+      <c r="B72" s="85"/>
       <c r="C72" s="53">
         <v>19.3</v>
       </c>
       <c r="D72" s="54" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="E72" s="54" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="F72" s="54" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="G72" s="55" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="H72" s="56"/>
       <c r="I72" s="57" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
     </row>
     <row r="73" spans="1:12" s="6" customFormat="1" ht="201.6" x14ac:dyDescent="0.3">
-      <c r="A73" s="58">
+      <c r="A73" s="80">
         <v>20</v>
       </c>
-      <c r="B73" s="61" t="s">
-        <v>130</v>
+      <c r="B73" s="83" t="s">
+        <v>126</v>
       </c>
       <c r="C73" s="44">
         <v>20.100000000000001</v>
       </c>
       <c r="D73" s="45" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="E73" s="45" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="F73" s="45" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="G73" s="46" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="H73" s="44"/>
       <c r="I73" s="47"/>
     </row>
     <row r="74" spans="1:12" s="6" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A74" s="59"/>
-      <c r="B74" s="62"/>
+      <c r="A74" s="81"/>
+      <c r="B74" s="84"/>
       <c r="C74" s="15">
         <v>20.2</v>
       </c>
       <c r="D74" s="45" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="E74" s="45" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="F74" s="45" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="G74" s="46" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="H74" s="44"/>
       <c r="I74" s="47"/>
@@ -7918,26 +7916,26 @@
       <c r="L74" s="1"/>
     </row>
     <row r="75" spans="1:12" s="6" customFormat="1" ht="283.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="60"/>
-      <c r="B75" s="62"/>
+      <c r="A75" s="82"/>
+      <c r="B75" s="84"/>
       <c r="C75" s="56">
         <v>20.3</v>
       </c>
       <c r="D75" s="54" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="E75" s="54" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="F75" s="54" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="G75" s="55" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="H75" s="56"/>
       <c r="I75" s="57" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="J75" s="1"/>
       <c r="K75" s="1"/>
@@ -7945,85 +7943,85 @@
     </row>
     <row r="76" spans="1:12" s="6" customFormat="1" ht="213" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="49"/>
-      <c r="B76" s="63"/>
+      <c r="B76" s="85"/>
       <c r="C76" s="56"/>
       <c r="D76" s="54" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="E76" s="54" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="F76" s="54" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="G76" s="55" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="H76" s="56"/>
       <c r="I76" s="57" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="J76" s="1"/>
       <c r="K76" s="1"/>
       <c r="L76" s="1"/>
     </row>
     <row r="77" spans="1:12" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="A77" s="58">
+      <c r="A77" s="80">
         <v>21</v>
       </c>
-      <c r="B77" s="61" t="s">
-        <v>133</v>
+      <c r="B77" s="83" t="s">
+        <v>129</v>
       </c>
       <c r="C77" s="44">
         <v>21.1</v>
       </c>
       <c r="D77" s="45" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="E77" s="45" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="F77" s="45" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="G77" s="46" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="H77" s="44"/>
       <c r="I77" s="47"/>
     </row>
     <row r="78" spans="1:12" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A78" s="59"/>
-      <c r="B78" s="62"/>
+      <c r="A78" s="81"/>
+      <c r="B78" s="84"/>
       <c r="C78" s="15">
         <v>21.2</v>
       </c>
       <c r="D78" s="45" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="E78" s="45" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="F78" s="45" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="G78" s="46" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="H78" s="44"/>
       <c r="I78" s="47"/>
     </row>
     <row r="79" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A79" s="60"/>
-      <c r="B79" s="63"/>
+      <c r="A79" s="82"/>
+      <c r="B79" s="85"/>
       <c r="C79" s="32">
         <v>21.3</v>
       </c>
       <c r="D79" s="16" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="E79" s="16" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="F79" s="16"/>
       <c r="G79" s="17"/>
@@ -8031,62 +8029,62 @@
       <c r="I79" s="33"/>
     </row>
     <row r="80" spans="1:12" ht="259.2" x14ac:dyDescent="0.3">
-      <c r="A80" s="58">
+      <c r="A80" s="80">
         <v>22</v>
       </c>
-      <c r="B80" s="61" t="s">
-        <v>137</v>
+      <c r="B80" s="83" t="s">
+        <v>133</v>
       </c>
       <c r="C80" s="44">
         <v>22.1</v>
       </c>
       <c r="D80" s="45" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="E80" s="45" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="F80" s="45" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="G80" s="46" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="H80" s="44"/>
       <c r="I80" s="47"/>
     </row>
     <row r="81" spans="1:9" ht="259.2" x14ac:dyDescent="0.3">
-      <c r="A81" s="59"/>
-      <c r="B81" s="62"/>
+      <c r="A81" s="81"/>
+      <c r="B81" s="84"/>
       <c r="C81" s="15">
         <v>22.2</v>
       </c>
       <c r="D81" s="45" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="E81" s="44" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="F81" s="45" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="G81" s="46" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="H81" s="44"/>
       <c r="I81" s="47"/>
     </row>
     <row r="82" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A82" s="60"/>
-      <c r="B82" s="63"/>
+      <c r="A82" s="82"/>
+      <c r="B82" s="85"/>
       <c r="C82" s="32">
         <v>22.3</v>
       </c>
       <c r="D82" s="16" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="E82" s="32" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="F82" s="16"/>
       <c r="G82" s="17"/>
@@ -8194,29 +8192,6 @@
   </sheetData>
   <autoFilter ref="I1:I32" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="37">
-    <mergeCell ref="A16:A19"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A46:A53"/>
-    <mergeCell ref="B46:B53"/>
-    <mergeCell ref="A30:A34"/>
-    <mergeCell ref="B30:B34"/>
-    <mergeCell ref="A35:A45"/>
-    <mergeCell ref="B35:B45"/>
-    <mergeCell ref="A27:A29"/>
-    <mergeCell ref="B27:B29"/>
-    <mergeCell ref="B16:B21"/>
-    <mergeCell ref="B22:B26"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="A11:A15"/>
-    <mergeCell ref="B11:B15"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:F1"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="A3:A7"/>
-    <mergeCell ref="B3:B10"/>
     <mergeCell ref="A77:A79"/>
     <mergeCell ref="B77:B79"/>
     <mergeCell ref="A80:A82"/>
@@ -8231,6 +8206,29 @@
     <mergeCell ref="A73:A75"/>
     <mergeCell ref="B73:B76"/>
     <mergeCell ref="B65:B69"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="A11:A15"/>
+    <mergeCell ref="B11:B15"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="A3:A7"/>
+    <mergeCell ref="B3:B10"/>
+    <mergeCell ref="A16:A19"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A46:A53"/>
+    <mergeCell ref="B46:B53"/>
+    <mergeCell ref="A30:A34"/>
+    <mergeCell ref="B30:B34"/>
+    <mergeCell ref="A35:A45"/>
+    <mergeCell ref="B35:B45"/>
+    <mergeCell ref="A27:A29"/>
+    <mergeCell ref="B27:B29"/>
+    <mergeCell ref="B16:B21"/>
+    <mergeCell ref="B22:B26"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8291,7 +8289,7 @@
         <v>8</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="I3" s="12" t="s">
         <v>4</v>
@@ -8303,22 +8301,22 @@
       <c r="B4" s="9"/>
       <c r="C4" s="9"/>
       <c r="D4" s="13" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E4" s="13">
         <v>14.1</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="I4" s="13" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="J4" s="9"/>
     </row>
@@ -8327,22 +8325,22 @@
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
       <c r="D5" s="13" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E5" s="13">
         <v>14.2</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="I5" s="13" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="J5" s="9"/>
     </row>
@@ -8351,22 +8349,22 @@
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
       <c r="D6" s="13" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E6" s="13">
         <v>14.3</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="I6" s="13" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="J6" s="9"/>
     </row>
@@ -8375,22 +8373,22 @@
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
       <c r="D7" s="13" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E7" s="13">
         <v>14.4</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="I7" s="13" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="J7" s="9"/>
     </row>
@@ -8399,22 +8397,22 @@
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
       <c r="D8" s="13" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E8" s="13">
         <v>14.5</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="I8" s="13" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="J8" s="9"/>
     </row>
@@ -8423,22 +8421,22 @@
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
       <c r="D9" s="13" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E9" s="13">
         <v>14.6</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="I9" s="13" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="J9" s="9"/>
     </row>
@@ -8447,22 +8445,22 @@
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
       <c r="D10" s="13" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E10" s="13">
         <v>14.7</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="I10" s="13" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="J10" s="9"/>
     </row>
@@ -8471,22 +8469,22 @@
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
       <c r="D11" s="13" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E11" s="13">
         <v>14.8</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="I11" s="13" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="J11" s="9"/>
     </row>
@@ -8495,22 +8493,22 @@
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
       <c r="D12" s="13" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E12" s="13">
         <v>14.9</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="I12" s="13" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="J12" s="9"/>
     </row>
@@ -8519,22 +8517,22 @@
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
       <c r="D13" s="13" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="I13" s="13" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="J13" s="9"/>
     </row>
@@ -8543,22 +8541,22 @@
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
       <c r="D14" s="13" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E14" s="13">
         <v>14.11</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="I14" s="13" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="J14" s="9"/>
     </row>

</xml_diff>

<commit_message>
Updated new acceptance criterion
</commit_message>
<xml_diff>
--- a/Business Analysis/checkupp_product_backlog.xlsx
+++ b/Business Analysis/checkupp_product_backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\CheckUpp\Business Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC7F28F7-BD9A-4F0F-808E-8B7A5B8CE6F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34550AD7-EA1C-44F2-8B37-D1E9B7DFAAAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5185,11 +5185,86 @@
     <t>I can quickly log my blood glucose level and assign it to the correct time of day.</t>
   </si>
   <si>
+    <t>Sprint 2</t>
+  </si>
+  <si>
+    <t>tap on a dedicated download option directly from the document card</t>
+  </si>
+  <si>
+    <t>I can save the document to my local device storage without having to open it first</t>
+  </si>
+  <si>
+    <t>1. If a document cannot be opened, an appropriate error message ('Could not open file') must be displayed, and the user must be able to retry opening the document.
+2. The selected document must be displayed in a readable format using the device's supported document viewer (Drive PDF Viewer, OneDrive PDF viewer, Adobe Acrobat Reader etc).
+3. The explicit "Download" button must be removed from this view screen, as it is now an independent card action.</t>
+  </si>
+  <si>
+    <t>access document actions through an organized card layout with an overflow menu</t>
+  </si>
+  <si>
+    <t>the interface remains uncluttered and accidental deletions are prevented</t>
+  </si>
+  <si>
+    <t>access link actions through a responsive card layout</t>
+  </si>
+  <si>
+    <t>the interface remains uncluttered regardless of my device's screen size</t>
+  </si>
+  <si>
+    <t>1. The logged-in user must be able to select one or more health documents (e.g., reports) from their local device for upload to the Document Wallet.
+2. The selected health documents must be uploaded securely to the app's Firebase Storage and associated with the logged-in user's account.
+3. A confirmation message must be displayed to the user after each document has been successfully uploaded.
+4. If a document upload fails, an appropriate error message must be displayed, and the user must be able to retry the upload without affecting previously uploaded documents.
+5. Document wallet must list all the uploaded documents with name and date.
+6. User must be able to interact with the options to download, view and delete options for each document stored in the Document Wallet.</t>
+  </si>
+  <si>
+    <t>1. User must be able to select the Delete option for any document stored in the Documents section of the Document Wallet.
+2. A confirmation prompt (Are you sure you want to delete this file?) must be displayed before the selected document is permanently deleted from Firebase Storage and the database.
+3. The selected document must be permanently removed from the logged-in user's Document Wallet and Firebase Storage after the deletion is confirmed.
+4. The deleted document must no longer be visible or accessible in the Document Wallet after successful deletion.
+5. If the document cannot be deleted, an appropriate error message (File could not be deleted, please try again) must be displayed, and the document must remain available in the Document Wallet until the deletion is successfully completed.</t>
+  </si>
+  <si>
+    <t>1. User must be able to initiate a download by tapping the Download option within the expanded 3-dot (kebab) action menu.
+2. The document must securely download to the user's local device storage.
+3. A success message (e.g., "Download complete") must be displayed upon completion.
+4. If the download fails, an error message must prompt the user to try again.</t>
+  </si>
+  <si>
+    <t>view (open inside app) a document stored in my document wallet</t>
+  </si>
+  <si>
+    <t>1. To prevent UI clutter on small devices, the card must display a standalone icon for "Share" alongside a vertical three-dot (kebab) menu.
+2. Expanding the kebab menu must reveal the "View", "Download", and "Delete" options.</t>
+  </si>
+  <si>
+    <t>1. User must be able to add an e-script link along with the associated text description of their choice in the Links section of the Document Wallet.
+2. All saved e-script links and their associated descriptions must be securely saved in the database and displayed as a list in the Links section.
+3. If an e-script link cannot be saved, an appropriate error message (Link could not be saved, Try again) must be displayed, and the user must be able to retry the action without affecting previously saved links.
+4. Document wallet must list all the saved links with name and date.
+5. User must be able to interact with standalone or menu-grouped options to open, share, and delete each link.</t>
+  </si>
+  <si>
+    <t>1. User must be able to select the Delete option for any e-script link stored in the Links section of the Document Wallet.
+2. A confirmation prompt (e.g., "Are you sure you want to delete this link?") must be displayed before the selected e-script link is permanently deleted from the database.
+3. The selected e-script link must be permanently removed from the logged-in user's Document Wallet and the database after the deletion is confirmed.
+4. The deleted e-script link must no longer be visible or accessible in the Links section after successful deletion.
+5. If the e-script link cannot be deleted, an appropriate error message (e.g., "Link could not be deleted, please try again.") must be displayed, and the link must remain available in the Document Wallet until the deletion is successfully completed.</t>
+  </si>
+  <si>
+    <t>1. The link card must display the "Share" icon alongside a vertical three-dot (kebab) menu to maintain consistency with the Documents tab.
+2. Expanding the kebab menu must reveal the "Open" and "Delete" options.</t>
+  </si>
+  <si>
     <t>1. Trigger: A "Scan Scale" icon next to the Weight input field (found in Diabetes and other modules).
 2. Extraction Logic: The ML Kit uses regex to capture a 2-to-3 digit number (with or without a single decimal, e.g., 75.4 or 98).
 3. Auto-Fill Execution: Automatically populates the Weight (kg) field. No secondary context modal is required (unlike the glucometer).
 4. Lighting/Contrast Pre-Processing (Technical AC): Because floor scales are often highly reflective or backlit, the camera feed passed to ML Kit must utilize a threshold/contrast filter to isolate the glowing LCD numbers from the background glare.
-5. Scan Timeout: If the ML Kit fails to detect valid text matching the required Regex patterns within 10 seconds of the camera opening, the app must show a prompt: "Having trouble reading the screen. Ensure there is no glare, or switch to manual entry." with an easy button to exit the camera view.</t>
+5. Scan Timeout: If the ML Kit fails to detect valid text matching the required Regex patterns within 10 seconds of the camera opening, the app must show a prompt: "Having trouble reading the screen. Ensure there is no glare, or switch to manual entry." with an easy button to exit the camera view.
+6. Multi-Frame Verification: The extraction logic must require the OCR engine to detect the exact same numeric reading across at least 2 to 3 consecutive camera frames before locking on and triggering the auto-fill, preventing errors caused by momentary screen glare or motion blur.
+7. Torch Toggle: A flashlight/torch toggle button must be available directly on the camera scan interface for low-light environments.
+8. Zero Network Dependency (Privacy): Because scanning runs strictly via on-device ML Kit, the extraction feature must operate flawlessly when the device is fully offline, ensuring no visual data is transmitted over the internet.</t>
   </si>
   <si>
     <t>1. Trigger: A single "Scan Glucometer" button must be available at the top of the Blood Glucose section in the Diabetes form.
@@ -5201,7 +5276,11 @@
 - Button 3: Post-Meal Glucose
 5. Auto-Fill Execution: Tapping one of the options closes the modal and injects the scanned number specifically into the chosen field.
 6. Validation: Same human-in-the-loop requirement. The user must manually click "Save Reading" at the bottom of the screen to commit to the database.
-7. Scan Timeout: If the ML Kit fails to detect valid text matching the required Regex patterns within 10 seconds of the camera opening, the app must show a prompt: "Having trouble reading the screen. Ensure there is no glare, or switch to manual entry." with an easy button to exit the camera view.</t>
+7. Scan Timeout: If the ML Kit fails to detect valid text matching the required Regex patterns within 10 seconds of the camera opening, the app must show a prompt: "Having trouble reading the screen. Ensure there is no glare, or switch to manual entry." with an easy button to exit the camera view.
+8. Multi-Frame Verification: The extraction logic must require the OCR engine to detect the exact same numeric reading across at least 2 to 3 consecutive camera frames before locking on and triggering the auto-fill, preventing errors caused by momentary screen glare or motion blur.
+9. Torch Toggle: A flashlight/torch toggle button must be available directly on the camera scan interface for low-light environments.
+10. Zero Network Dependency (Privacy): Because scanning runs strictly via on-device ML Kit, the extraction feature must operate flawlessly when the device is fully offline, ensuring no visual data is transmitted over the internet.
+11. Lighting/Contrast Pre-Processing (Technical AC): Because floor scales are often highly reflective or backlit, the camera feed passed to ML Kit must utilize a threshold/contrast filter to isolate the glowing LCD numbers from the background glare.</t>
   </si>
   <si>
     <t>1. Trigger: A "Scan Monitor" icon/button must be visible next to the manual input fields for Blood Pressure in the Cardiovascular Health form.
@@ -5214,79 +5293,11 @@
 - Lowest Y-coordinate = Auto-fills Heart Rate (BPM)
 6. Human-in-the-Loop Validation: Upon successful extraction, the camera closes, the fields populate, and a Toast/Banner must display: "Numbers scanned successfully. Please verify against your device."
 7. Fallback: A manual "Cancel/Enter Manually" button must always be present on the camera screen.
-8. Scan Timeout: If the ML Kit fails to detect valid text matching the required Regex patterns within 10 seconds of the camera opening, the app must show a prompt: "Having trouble reading the screen. Ensure there is no glare, or switch to manual entry." with an easy button to exit the camera view.</t>
-  </si>
-  <si>
-    <t>Sprint 2</t>
-  </si>
-  <si>
-    <t>tap on a dedicated download option directly from the document card</t>
-  </si>
-  <si>
-    <t>I can save the document to my local device storage without having to open it first</t>
-  </si>
-  <si>
-    <t>1. If a document cannot be opened, an appropriate error message ('Could not open file') must be displayed, and the user must be able to retry opening the document.
-2. The selected document must be displayed in a readable format using the device's supported document viewer (Drive PDF Viewer, OneDrive PDF viewer, Adobe Acrobat Reader etc).
-3. The explicit "Download" button must be removed from this view screen, as it is now an independent card action.</t>
-  </si>
-  <si>
-    <t>access document actions through an organized card layout with an overflow menu</t>
-  </si>
-  <si>
-    <t>the interface remains uncluttered and accidental deletions are prevented</t>
-  </si>
-  <si>
-    <t>access link actions through a responsive card layout</t>
-  </si>
-  <si>
-    <t>the interface remains uncluttered regardless of my device's screen size</t>
-  </si>
-  <si>
-    <t>1. The logged-in user must be able to select one or more health documents (e.g., reports) from their local device for upload to the Document Wallet.
-2. The selected health documents must be uploaded securely to the app's Firebase Storage and associated with the logged-in user's account.
-3. A confirmation message must be displayed to the user after each document has been successfully uploaded.
-4. If a document upload fails, an appropriate error message must be displayed, and the user must be able to retry the upload without affecting previously uploaded documents.
-5. Document wallet must list all the uploaded documents with name and date.
-6. User must be able to interact with the options to download, view and delete options for each document stored in the Document Wallet.</t>
-  </si>
-  <si>
-    <t>1. User must be able to select the Delete option for any document stored in the Documents section of the Document Wallet.
-2. A confirmation prompt (Are you sure you want to delete this file?) must be displayed before the selected document is permanently deleted from Firebase Storage and the database.
-3. The selected document must be permanently removed from the logged-in user's Document Wallet and Firebase Storage after the deletion is confirmed.
-4. The deleted document must no longer be visible or accessible in the Document Wallet after successful deletion.
-5. If the document cannot be deleted, an appropriate error message (File could not be deleted, please try again) must be displayed, and the document must remain available in the Document Wallet until the deletion is successfully completed.</t>
-  </si>
-  <si>
-    <t>1. User must be able to initiate a download by tapping the Download option within the expanded 3-dot (kebab) action menu.
-2. The document must securely download to the user's local device storage.
-3. A success message (e.g., "Download complete") must be displayed upon completion.
-4. If the download fails, an error message must prompt the user to try again.</t>
-  </si>
-  <si>
-    <t>view (open inside app) a document stored in my document wallet</t>
-  </si>
-  <si>
-    <t>1. To prevent UI clutter on small devices, the card must display a standalone icon for "Share" alongside a vertical three-dot (kebab) menu.
-2. Expanding the kebab menu must reveal the "View", "Download", and "Delete" options.</t>
-  </si>
-  <si>
-    <t>1. User must be able to add an e-script link along with the associated text description of their choice in the Links section of the Document Wallet.
-2. All saved e-script links and their associated descriptions must be securely saved in the database and displayed as a list in the Links section.
-3. If an e-script link cannot be saved, an appropriate error message (Link could not be saved, Try again) must be displayed, and the user must be able to retry the action without affecting previously saved links.
-4. Document wallet must list all the saved links with name and date.
-5. User must be able to interact with standalone or menu-grouped options to open, share, and delete each link.</t>
-  </si>
-  <si>
-    <t>1. User must be able to select the Delete option for any e-script link stored in the Links section of the Document Wallet.
-2. A confirmation prompt (e.g., "Are you sure you want to delete this link?") must be displayed before the selected e-script link is permanently deleted from the database.
-3. The selected e-script link must be permanently removed from the logged-in user's Document Wallet and the database after the deletion is confirmed.
-4. The deleted e-script link must no longer be visible or accessible in the Links section after successful deletion.
-5. If the e-script link cannot be deleted, an appropriate error message (e.g., "Link could not be deleted, please try again.") must be displayed, and the link must remain available in the Document Wallet until the deletion is successfully completed.</t>
-  </si>
-  <si>
-    <t>1. The link card must display the "Share" icon alongside a vertical three-dot (kebab) menu to maintain consistency with the Documents tab.
-2. Expanding the kebab menu must reveal the "Open" and "Delete" options.</t>
+8. Scan Timeout: If the ML Kit fails to detect valid text matching the required Regex patterns within 10 seconds of the camera opening, the app must show a prompt: "Having trouble reading the screen. Ensure there is no glare, or switch to manual entry." with an easy button to exit the camera view.
+9. Multi-Frame Verification: The extraction logic must require the OCR engine to detect the exact same numeric reading across at least 2 to 3 consecutive camera frames before locking on and triggering the auto-fill, preventing errors caused by momentary screen glare or motion blur.
+10. Torch Toggle: A flashlight/torch toggle button must be available directly on the camera scan interface for low-light environments.
+11. Zero Network Dependency (Privacy): Because scanning runs strictly via on-device ML Kit, the extraction feature must operate flawlessly when the device is fully offline, ensuring no visual data is transmitted over the internet.
+12. Lighting/Contrast Pre-Processing (Technical AC): Because floor scales are often highly reflective or backlit, the camera feed passed to ML Kit must utilize a threshold/contrast filter to isolate the glowing LCD numbers from the background glare.</t>
   </si>
 </sst>
 </file>
@@ -5786,6 +5797,72 @@
     <xf numFmtId="0" fontId="2" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -5804,9 +5881,6 @@
     <xf numFmtId="0" fontId="15" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -5823,69 +5897,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6121,34 +6132,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="71" t="s">
+      <c r="A1" s="74" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="71" t="s">
+      <c r="B1" s="74" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="71" t="s">
+      <c r="C1" s="74" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="71" t="s">
+      <c r="D1" s="74" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
+      <c r="E1" s="65"/>
+      <c r="F1" s="65"/>
       <c r="G1" s="75" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="71" t="s">
+      <c r="H1" s="74" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="71" t="s">
+      <c r="I1" s="74" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="64"/>
-      <c r="B2" s="64"/>
-      <c r="C2" s="64"/>
+      <c r="A2" s="65"/>
+      <c r="B2" s="65"/>
+      <c r="C2" s="65"/>
       <c r="D2" s="4" t="s">
         <v>7</v>
       </c>
@@ -6159,8 +6170,8 @@
         <v>9</v>
       </c>
       <c r="G2" s="75"/>
-      <c r="H2" s="64"/>
-      <c r="I2" s="64"/>
+      <c r="H2" s="65"/>
+      <c r="I2" s="65"/>
     </row>
     <row r="3" spans="1:9" s="5" customFormat="1" ht="108" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="76">
@@ -6339,10 +6350,10 @@
       <c r="I10" s="51"/>
     </row>
     <row r="11" spans="1:9" s="6" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="72">
+      <c r="A11" s="71">
         <v>5</v>
       </c>
-      <c r="B11" s="72" t="s">
+      <c r="B11" s="71" t="s">
         <v>13</v>
       </c>
       <c r="C11" s="18">
@@ -6368,8 +6379,8 @@
       </c>
     </row>
     <row r="12" spans="1:9" s="6" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="73"/>
-      <c r="B12" s="73"/>
+      <c r="A12" s="72"/>
+      <c r="B12" s="72"/>
       <c r="C12" s="18">
         <v>5.2</v>
       </c>
@@ -6389,8 +6400,8 @@
       <c r="I12" s="18"/>
     </row>
     <row r="13" spans="1:9" s="6" customFormat="1" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="73"/>
-      <c r="B13" s="73"/>
+      <c r="A13" s="72"/>
+      <c r="B13" s="72"/>
       <c r="C13" s="18">
         <v>5.3</v>
       </c>
@@ -6410,8 +6421,8 @@
       <c r="I13" s="18"/>
     </row>
     <row r="14" spans="1:9" s="14" customFormat="1" ht="230.4" x14ac:dyDescent="0.3">
-      <c r="A14" s="73"/>
-      <c r="B14" s="73"/>
+      <c r="A14" s="72"/>
+      <c r="B14" s="72"/>
       <c r="C14" s="21">
         <v>5.4</v>
       </c>
@@ -6431,8 +6442,8 @@
       <c r="I14" s="21"/>
     </row>
     <row r="15" spans="1:9" s="14" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A15" s="74"/>
-      <c r="B15" s="74"/>
+      <c r="A15" s="73"/>
+      <c r="B15" s="73"/>
       <c r="C15" s="21">
         <v>5.5</v>
       </c>
@@ -6452,10 +6463,10 @@
       <c r="I15" s="21"/>
     </row>
     <row r="16" spans="1:9" s="14" customFormat="1" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="58">
+      <c r="A16" s="80">
         <v>6</v>
       </c>
-      <c r="B16" s="58" t="s">
+      <c r="B16" s="80" t="s">
         <v>25</v>
       </c>
       <c r="C16" s="24">
@@ -6471,7 +6482,7 @@
         <v>28</v>
       </c>
       <c r="G16" s="25" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="H16" s="26" t="s">
         <v>29</v>
@@ -6481,8 +6492,8 @@
       </c>
     </row>
     <row r="17" spans="1:9" s="6" customFormat="1" ht="144" x14ac:dyDescent="0.3">
-      <c r="A17" s="59"/>
-      <c r="B17" s="59"/>
+      <c r="A17" s="81"/>
+      <c r="B17" s="81"/>
       <c r="C17" s="24">
         <v>6.2</v>
       </c>
@@ -6502,8 +6513,8 @@
       <c r="I17" s="24"/>
     </row>
     <row r="18" spans="1:9" s="6" customFormat="1" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="59"/>
-      <c r="B18" s="59"/>
+      <c r="A18" s="81"/>
+      <c r="B18" s="81"/>
       <c r="C18" s="24">
         <v>6.3</v>
       </c>
@@ -6517,14 +6528,14 @@
         <v>32</v>
       </c>
       <c r="G18" s="25" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="H18" s="26"/>
       <c r="I18" s="24"/>
     </row>
     <row r="19" spans="1:9" s="6" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A19" s="59"/>
-      <c r="B19" s="59"/>
+      <c r="A19" s="81"/>
+      <c r="B19" s="81"/>
       <c r="C19" s="27">
         <v>6.4</v>
       </c>
@@ -6532,13 +6543,13 @@
         <v>26</v>
       </c>
       <c r="E19" s="24" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="F19" s="24" t="s">
         <v>33</v>
       </c>
       <c r="G19" s="25" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="H19" s="26" t="s">
         <v>29</v>
@@ -6549,7 +6560,7 @@
     </row>
     <row r="20" spans="1:9" s="6" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A20" s="52"/>
-      <c r="B20" s="59"/>
+      <c r="B20" s="81"/>
       <c r="C20" s="24">
         <v>6.5</v>
       </c>
@@ -6557,20 +6568,20 @@
         <v>26</v>
       </c>
       <c r="E20" s="24" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="F20" s="24" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="G20" s="25" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="H20" s="26"/>
       <c r="I20" s="24"/>
     </row>
     <row r="21" spans="1:9" s="6" customFormat="1" ht="72" x14ac:dyDescent="0.3">
       <c r="A21" s="52"/>
-      <c r="B21" s="70"/>
+      <c r="B21" s="91"/>
       <c r="C21" s="24">
         <v>6.6</v>
       </c>
@@ -6578,22 +6589,22 @@
         <v>26</v>
       </c>
       <c r="E21" s="24" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="F21" s="24" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="G21" s="25" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="H21" s="26"/>
       <c r="I21" s="24"/>
     </row>
     <row r="22" spans="1:9" s="6" customFormat="1" ht="144" x14ac:dyDescent="0.3">
-      <c r="A22" s="60">
+      <c r="A22" s="82">
         <v>7</v>
       </c>
-      <c r="B22" s="58" t="s">
+      <c r="B22" s="80" t="s">
         <v>34</v>
       </c>
       <c r="C22" s="24">
@@ -6609,7 +6620,7 @@
         <v>37</v>
       </c>
       <c r="G22" s="25" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="H22" s="26" t="s">
         <v>29</v>
@@ -6619,8 +6630,8 @@
       </c>
     </row>
     <row r="23" spans="1:9" s="6" customFormat="1" ht="72" x14ac:dyDescent="0.3">
-      <c r="A23" s="61"/>
-      <c r="B23" s="59"/>
+      <c r="A23" s="83"/>
+      <c r="B23" s="81"/>
       <c r="C23" s="24">
         <v>7.2</v>
       </c>
@@ -6642,8 +6653,8 @@
       </c>
     </row>
     <row r="24" spans="1:9" s="6" customFormat="1" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="A24" s="61"/>
-      <c r="B24" s="59"/>
+      <c r="A24" s="83"/>
+      <c r="B24" s="81"/>
       <c r="C24" s="24">
         <v>7.3</v>
       </c>
@@ -6663,8 +6674,8 @@
       <c r="I24" s="24"/>
     </row>
     <row r="25" spans="1:9" s="6" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A25" s="62"/>
-      <c r="B25" s="59"/>
+      <c r="A25" s="84"/>
+      <c r="B25" s="81"/>
       <c r="C25" s="24">
         <v>7.4</v>
       </c>
@@ -6678,14 +6689,14 @@
         <v>43</v>
       </c>
       <c r="G25" s="25" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="H25" s="26"/>
       <c r="I25" s="24"/>
     </row>
     <row r="26" spans="1:9" s="6" customFormat="1" ht="72" x14ac:dyDescent="0.3">
       <c r="A26" s="52"/>
-      <c r="B26" s="70"/>
+      <c r="B26" s="91"/>
       <c r="C26" s="24">
         <v>7.5</v>
       </c>
@@ -6693,22 +6704,22 @@
         <v>35</v>
       </c>
       <c r="E26" s="24" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="F26" s="24" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="G26" s="25" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="H26" s="26"/>
       <c r="I26" s="24"/>
     </row>
     <row r="27" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A27" s="67">
+      <c r="A27" s="88">
         <v>8</v>
       </c>
-      <c r="B27" s="67" t="s">
+      <c r="B27" s="88" t="s">
         <v>44</v>
       </c>
       <c r="C27" s="28">
@@ -6732,8 +6743,8 @@
       </c>
     </row>
     <row r="28" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A28" s="68"/>
-      <c r="B28" s="68"/>
+      <c r="A28" s="89"/>
+      <c r="B28" s="89"/>
       <c r="C28" s="28">
         <v>9.3000000000000007</v>
       </c>
@@ -6755,8 +6766,8 @@
       </c>
     </row>
     <row r="29" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A29" s="69"/>
-      <c r="B29" s="69"/>
+      <c r="A29" s="90"/>
+      <c r="B29" s="90"/>
       <c r="C29" s="28">
         <v>9.4</v>
       </c>
@@ -6778,10 +6789,10 @@
       </c>
     </row>
     <row r="30" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="65">
+      <c r="A30" s="86">
         <v>12</v>
       </c>
-      <c r="B30" s="65" t="s">
+      <c r="B30" s="86" t="s">
         <v>54</v>
       </c>
       <c r="C30" s="30">
@@ -6807,8 +6818,8 @@
       </c>
     </row>
     <row r="31" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A31" s="65"/>
-      <c r="B31" s="65"/>
+      <c r="A31" s="86"/>
+      <c r="B31" s="86"/>
       <c r="C31" s="30">
         <v>12.2</v>
       </c>
@@ -6832,8 +6843,8 @@
       </c>
     </row>
     <row r="32" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="65"/>
-      <c r="B32" s="65"/>
+      <c r="A32" s="86"/>
+      <c r="B32" s="86"/>
       <c r="C32" s="30">
         <v>12.3</v>
       </c>
@@ -6857,8 +6868,8 @@
       </c>
     </row>
     <row r="33" spans="1:9" s="6" customFormat="1" ht="123.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="65"/>
-      <c r="B33" s="65"/>
+      <c r="A33" s="86"/>
+      <c r="B33" s="86"/>
       <c r="C33" s="30">
         <v>12.4</v>
       </c>
@@ -6882,8 +6893,8 @@
       </c>
     </row>
     <row r="34" spans="1:9" s="6" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A34" s="65"/>
-      <c r="B34" s="65"/>
+      <c r="A34" s="86"/>
+      <c r="B34" s="86"/>
       <c r="C34" s="30">
         <v>12.5</v>
       </c>
@@ -6907,10 +6918,10 @@
       </c>
     </row>
     <row r="35" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A35" s="66">
+      <c r="A35" s="87">
         <v>14</v>
       </c>
-      <c r="B35" s="66" t="s">
+      <c r="B35" s="87" t="s">
         <v>70</v>
       </c>
       <c r="C35" s="34">
@@ -6936,8 +6947,8 @@
       </c>
     </row>
     <row r="36" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A36" s="66"/>
-      <c r="B36" s="66"/>
+      <c r="A36" s="87"/>
+      <c r="B36" s="87"/>
       <c r="C36" s="34">
         <v>14.2</v>
       </c>
@@ -6961,8 +6972,8 @@
       </c>
     </row>
     <row r="37" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A37" s="66"/>
-      <c r="B37" s="66"/>
+      <c r="A37" s="87"/>
+      <c r="B37" s="87"/>
       <c r="C37" s="34">
         <v>14.3</v>
       </c>
@@ -6986,8 +6997,8 @@
       </c>
     </row>
     <row r="38" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A38" s="66"/>
-      <c r="B38" s="66"/>
+      <c r="A38" s="87"/>
+      <c r="B38" s="87"/>
       <c r="C38" s="34">
         <v>14.4</v>
       </c>
@@ -7011,8 +7022,8 @@
       </c>
     </row>
     <row r="39" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A39" s="66"/>
-      <c r="B39" s="66"/>
+      <c r="A39" s="87"/>
+      <c r="B39" s="87"/>
       <c r="C39" s="34">
         <v>14.5</v>
       </c>
@@ -7036,8 +7047,8 @@
       </c>
     </row>
     <row r="40" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A40" s="66"/>
-      <c r="B40" s="66"/>
+      <c r="A40" s="87"/>
+      <c r="B40" s="87"/>
       <c r="C40" s="34">
         <v>14.6</v>
       </c>
@@ -7061,8 +7072,8 @@
       </c>
     </row>
     <row r="41" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A41" s="66"/>
-      <c r="B41" s="66"/>
+      <c r="A41" s="87"/>
+      <c r="B41" s="87"/>
       <c r="C41" s="34">
         <v>14.7</v>
       </c>
@@ -7086,8 +7097,8 @@
       </c>
     </row>
     <row r="42" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A42" s="66"/>
-      <c r="B42" s="66"/>
+      <c r="A42" s="87"/>
+      <c r="B42" s="87"/>
       <c r="C42" s="34">
         <v>14.8</v>
       </c>
@@ -7111,8 +7122,8 @@
       </c>
     </row>
     <row r="43" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A43" s="66"/>
-      <c r="B43" s="66"/>
+      <c r="A43" s="87"/>
+      <c r="B43" s="87"/>
       <c r="C43" s="34">
         <v>14.9</v>
       </c>
@@ -7136,8 +7147,8 @@
       </c>
     </row>
     <row r="44" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A44" s="66"/>
-      <c r="B44" s="66"/>
+      <c r="A44" s="87"/>
+      <c r="B44" s="87"/>
       <c r="C44" s="34">
         <v>14.1</v>
       </c>
@@ -7161,8 +7172,8 @@
       </c>
     </row>
     <row r="45" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A45" s="66"/>
-      <c r="B45" s="66"/>
+      <c r="A45" s="87"/>
+      <c r="B45" s="87"/>
       <c r="C45" s="34">
         <v>14.11</v>
       </c>
@@ -7186,10 +7197,10 @@
       </c>
     </row>
     <row r="46" spans="1:9" s="6" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A46" s="63">
+      <c r="A46" s="85">
         <v>15</v>
       </c>
-      <c r="B46" s="63" t="s">
+      <c r="B46" s="85" t="s">
         <v>74</v>
       </c>
       <c r="C46" s="37">
@@ -7215,8 +7226,8 @@
       </c>
     </row>
     <row r="47" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A47" s="64"/>
-      <c r="B47" s="64"/>
+      <c r="A47" s="65"/>
+      <c r="B47" s="65"/>
       <c r="C47" s="37">
         <v>15.2</v>
       </c>
@@ -7240,8 +7251,8 @@
       </c>
     </row>
     <row r="48" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A48" s="64"/>
-      <c r="B48" s="64"/>
+      <c r="A48" s="65"/>
+      <c r="B48" s="65"/>
       <c r="C48" s="37">
         <v>15.3</v>
       </c>
@@ -7265,8 +7276,8 @@
       </c>
     </row>
     <row r="49" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A49" s="64"/>
-      <c r="B49" s="64"/>
+      <c r="A49" s="65"/>
+      <c r="B49" s="65"/>
       <c r="C49" s="37">
         <v>15.4</v>
       </c>
@@ -7290,8 +7301,8 @@
       </c>
     </row>
     <row r="50" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A50" s="64"/>
-      <c r="B50" s="64"/>
+      <c r="A50" s="65"/>
+      <c r="B50" s="65"/>
       <c r="C50" s="37">
         <v>15.5</v>
       </c>
@@ -7315,8 +7326,8 @@
       </c>
     </row>
     <row r="51" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A51" s="64"/>
-      <c r="B51" s="64"/>
+      <c r="A51" s="65"/>
+      <c r="B51" s="65"/>
       <c r="C51" s="37">
         <v>15.6</v>
       </c>
@@ -7340,8 +7351,8 @@
       </c>
     </row>
     <row r="52" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A52" s="64"/>
-      <c r="B52" s="64"/>
+      <c r="A52" s="65"/>
+      <c r="B52" s="65"/>
       <c r="C52" s="37">
         <v>15.7</v>
       </c>
@@ -7365,8 +7376,8 @@
       </c>
     </row>
     <row r="53" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A53" s="64"/>
-      <c r="B53" s="64"/>
+      <c r="A53" s="65"/>
+      <c r="B53" s="65"/>
       <c r="C53" s="37">
         <v>15.8</v>
       </c>
@@ -7390,10 +7401,10 @@
       </c>
     </row>
     <row r="54" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A54" s="86">
+      <c r="A54" s="64">
         <v>16</v>
       </c>
-      <c r="B54" s="86" t="s">
+      <c r="B54" s="64" t="s">
         <v>89</v>
       </c>
       <c r="C54" s="39">
@@ -7419,8 +7430,8 @@
       </c>
     </row>
     <row r="55" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A55" s="86"/>
-      <c r="B55" s="86"/>
+      <c r="A55" s="64"/>
+      <c r="B55" s="64"/>
       <c r="C55" s="39">
         <v>16.2</v>
       </c>
@@ -7444,8 +7455,8 @@
       </c>
     </row>
     <row r="56" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A56" s="86"/>
-      <c r="B56" s="86"/>
+      <c r="A56" s="64"/>
+      <c r="B56" s="64"/>
       <c r="C56" s="39">
         <v>16.3</v>
       </c>
@@ -7469,8 +7480,8 @@
       </c>
     </row>
     <row r="57" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A57" s="86"/>
-      <c r="B57" s="86"/>
+      <c r="A57" s="64"/>
+      <c r="B57" s="64"/>
       <c r="C57" s="39">
         <v>16.399999999999999</v>
       </c>
@@ -7494,8 +7505,8 @@
       </c>
     </row>
     <row r="58" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A58" s="86"/>
-      <c r="B58" s="86"/>
+      <c r="A58" s="64"/>
+      <c r="B58" s="64"/>
       <c r="C58" s="39">
         <v>16.5</v>
       </c>
@@ -7519,8 +7530,8 @@
       </c>
     </row>
     <row r="59" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A59" s="64"/>
-      <c r="B59" s="64"/>
+      <c r="A59" s="65"/>
+      <c r="B59" s="65"/>
       <c r="C59" s="39">
         <v>16.600000000000001</v>
       </c>
@@ -7544,10 +7555,10 @@
       </c>
     </row>
     <row r="60" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A60" s="87">
+      <c r="A60" s="66">
         <v>17</v>
       </c>
-      <c r="B60" s="90" t="s">
+      <c r="B60" s="69" t="s">
         <v>105</v>
       </c>
       <c r="C60" s="42">
@@ -7573,8 +7584,8 @@
       </c>
     </row>
     <row r="61" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A61" s="88"/>
-      <c r="B61" s="90"/>
+      <c r="A61" s="67"/>
+      <c r="B61" s="69"/>
       <c r="C61" s="42">
         <v>17.2</v>
       </c>
@@ -7598,8 +7609,8 @@
       </c>
     </row>
     <row r="62" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A62" s="88"/>
-      <c r="B62" s="90"/>
+      <c r="A62" s="67"/>
+      <c r="B62" s="69"/>
       <c r="C62" s="42">
         <v>17.3</v>
       </c>
@@ -7623,8 +7634,8 @@
       </c>
     </row>
     <row r="63" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A63" s="88"/>
-      <c r="B63" s="90"/>
+      <c r="A63" s="67"/>
+      <c r="B63" s="69"/>
       <c r="C63" s="42">
         <v>17.399999999999999</v>
       </c>
@@ -7648,8 +7659,8 @@
       </c>
     </row>
     <row r="64" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A64" s="89"/>
-      <c r="B64" s="90"/>
+      <c r="A64" s="68"/>
+      <c r="B64" s="69"/>
       <c r="C64" s="42">
         <v>17.5</v>
       </c>
@@ -7673,10 +7684,10 @@
       </c>
     </row>
     <row r="65" spans="1:12" s="6" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A65" s="91">
+      <c r="A65" s="70">
         <v>18</v>
       </c>
-      <c r="B65" s="72" t="s">
+      <c r="B65" s="71" t="s">
         <v>279</v>
       </c>
       <c r="C65" s="18">
@@ -7702,8 +7713,8 @@
       </c>
     </row>
     <row r="66" spans="1:12" s="6" customFormat="1" ht="250.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="64"/>
-      <c r="B66" s="73"/>
+      <c r="A66" s="65"/>
+      <c r="B66" s="72"/>
       <c r="C66" s="18">
         <v>18.2</v>
       </c>
@@ -7727,8 +7738,8 @@
       </c>
     </row>
     <row r="67" spans="1:12" s="6" customFormat="1" ht="167.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="64"/>
-      <c r="B67" s="73"/>
+      <c r="A67" s="65"/>
+      <c r="B67" s="72"/>
       <c r="C67" s="18">
         <v>18.3</v>
       </c>
@@ -7752,8 +7763,8 @@
       </c>
     </row>
     <row r="68" spans="1:12" s="6" customFormat="1" ht="244.8" x14ac:dyDescent="0.3">
-      <c r="A68" s="64"/>
-      <c r="B68" s="73"/>
+      <c r="A68" s="65"/>
+      <c r="B68" s="72"/>
       <c r="C68" s="18">
         <v>18.399999999999999</v>
       </c>
@@ -7778,7 +7789,7 @@
     </row>
     <row r="69" spans="1:12" s="6" customFormat="1" ht="216" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="48"/>
-      <c r="B69" s="74"/>
+      <c r="B69" s="73"/>
       <c r="C69" s="18">
         <v>18.5</v>
       </c>
@@ -7798,10 +7809,10 @@
       <c r="I69" s="18"/>
     </row>
     <row r="70" spans="1:12" s="6" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A70" s="80">
+      <c r="A70" s="58">
         <v>19</v>
       </c>
-      <c r="B70" s="83" t="s">
+      <c r="B70" s="61" t="s">
         <v>120</v>
       </c>
       <c r="C70" s="44">
@@ -7823,8 +7834,8 @@
       <c r="I70" s="47"/>
     </row>
     <row r="71" spans="1:12" s="6" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A71" s="81"/>
-      <c r="B71" s="84"/>
+      <c r="A71" s="59"/>
+      <c r="B71" s="62"/>
       <c r="C71" s="15">
         <v>19.2</v>
       </c>
@@ -7843,9 +7854,9 @@
       <c r="H71" s="44"/>
       <c r="I71" s="47"/>
     </row>
-    <row r="72" spans="1:12" s="6" customFormat="1" ht="355.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="82"/>
-      <c r="B72" s="85"/>
+    <row r="72" spans="1:12" s="6" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A72" s="60"/>
+      <c r="B72" s="63"/>
       <c r="C72" s="53">
         <v>19.3</v>
       </c>
@@ -7859,18 +7870,18 @@
         <v>308</v>
       </c>
       <c r="G72" s="55" t="s">
-        <v>315</v>
+        <v>331</v>
       </c>
       <c r="H72" s="56"/>
       <c r="I72" s="57" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
     </row>
     <row r="73" spans="1:12" s="6" customFormat="1" ht="201.6" x14ac:dyDescent="0.3">
-      <c r="A73" s="80">
+      <c r="A73" s="58">
         <v>20</v>
       </c>
-      <c r="B73" s="83" t="s">
+      <c r="B73" s="61" t="s">
         <v>126</v>
       </c>
       <c r="C73" s="44">
@@ -7892,8 +7903,8 @@
       <c r="I73" s="47"/>
     </row>
     <row r="74" spans="1:12" s="6" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A74" s="81"/>
-      <c r="B74" s="84"/>
+      <c r="A74" s="59"/>
+      <c r="B74" s="62"/>
       <c r="C74" s="15">
         <v>20.2</v>
       </c>
@@ -7915,9 +7926,9 @@
       <c r="K74" s="1"/>
       <c r="L74" s="1"/>
     </row>
-    <row r="75" spans="1:12" s="6" customFormat="1" ht="283.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="82"/>
-      <c r="B75" s="84"/>
+    <row r="75" spans="1:12" s="6" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A75" s="60"/>
+      <c r="B75" s="62"/>
       <c r="C75" s="56">
         <v>20.3</v>
       </c>
@@ -7931,20 +7942,22 @@
         <v>312</v>
       </c>
       <c r="G75" s="55" t="s">
-        <v>314</v>
+        <v>330</v>
       </c>
       <c r="H75" s="56"/>
       <c r="I75" s="57" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="J75" s="1"/>
       <c r="K75" s="1"/>
       <c r="L75" s="1"/>
     </row>
-    <row r="76" spans="1:12" s="6" customFormat="1" ht="213" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:12" s="6" customFormat="1" ht="331.2" x14ac:dyDescent="0.3">
       <c r="A76" s="49"/>
-      <c r="B76" s="85"/>
-      <c r="C76" s="56"/>
+      <c r="B76" s="63"/>
+      <c r="C76" s="56">
+        <v>20.399999999999999</v>
+      </c>
       <c r="D76" s="54" t="s">
         <v>127</v>
       </c>
@@ -7955,21 +7968,21 @@
         <v>311</v>
       </c>
       <c r="G76" s="55" t="s">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="H76" s="56"/>
       <c r="I76" s="57" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="J76" s="1"/>
       <c r="K76" s="1"/>
       <c r="L76" s="1"/>
     </row>
     <row r="77" spans="1:12" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="A77" s="80">
+      <c r="A77" s="58">
         <v>21</v>
       </c>
-      <c r="B77" s="83" t="s">
+      <c r="B77" s="61" t="s">
         <v>129</v>
       </c>
       <c r="C77" s="44">
@@ -7991,8 +8004,8 @@
       <c r="I77" s="47"/>
     </row>
     <row r="78" spans="1:12" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A78" s="81"/>
-      <c r="B78" s="84"/>
+      <c r="A78" s="59"/>
+      <c r="B78" s="62"/>
       <c r="C78" s="15">
         <v>21.2</v>
       </c>
@@ -8012,8 +8025,8 @@
       <c r="I78" s="47"/>
     </row>
     <row r="79" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A79" s="82"/>
-      <c r="B79" s="85"/>
+      <c r="A79" s="60"/>
+      <c r="B79" s="63"/>
       <c r="C79" s="32">
         <v>21.3</v>
       </c>
@@ -8029,10 +8042,10 @@
       <c r="I79" s="33"/>
     </row>
     <row r="80" spans="1:12" ht="259.2" x14ac:dyDescent="0.3">
-      <c r="A80" s="80">
+      <c r="A80" s="58">
         <v>22</v>
       </c>
-      <c r="B80" s="83" t="s">
+      <c r="B80" s="61" t="s">
         <v>133</v>
       </c>
       <c r="C80" s="44">
@@ -8054,8 +8067,8 @@
       <c r="I80" s="47"/>
     </row>
     <row r="81" spans="1:9" ht="259.2" x14ac:dyDescent="0.3">
-      <c r="A81" s="81"/>
-      <c r="B81" s="84"/>
+      <c r="A81" s="59"/>
+      <c r="B81" s="62"/>
       <c r="C81" s="15">
         <v>22.2</v>
       </c>
@@ -8075,8 +8088,8 @@
       <c r="I81" s="47"/>
     </row>
     <row r="82" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A82" s="82"/>
-      <c r="B82" s="85"/>
+      <c r="A82" s="60"/>
+      <c r="B82" s="63"/>
       <c r="C82" s="32">
         <v>22.3</v>
       </c>
@@ -8192,6 +8205,29 @@
   </sheetData>
   <autoFilter ref="I1:I32" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="37">
+    <mergeCell ref="A16:A19"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A46:A53"/>
+    <mergeCell ref="B46:B53"/>
+    <mergeCell ref="A30:A34"/>
+    <mergeCell ref="B30:B34"/>
+    <mergeCell ref="A35:A45"/>
+    <mergeCell ref="B35:B45"/>
+    <mergeCell ref="A27:A29"/>
+    <mergeCell ref="B27:B29"/>
+    <mergeCell ref="B16:B21"/>
+    <mergeCell ref="B22:B26"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="A11:A15"/>
+    <mergeCell ref="B11:B15"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="A3:A7"/>
+    <mergeCell ref="B3:B10"/>
     <mergeCell ref="A77:A79"/>
     <mergeCell ref="B77:B79"/>
     <mergeCell ref="A80:A82"/>
@@ -8206,29 +8242,6 @@
     <mergeCell ref="A73:A75"/>
     <mergeCell ref="B73:B76"/>
     <mergeCell ref="B65:B69"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="A11:A15"/>
-    <mergeCell ref="B11:B15"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:F1"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="A3:A7"/>
-    <mergeCell ref="B3:B10"/>
-    <mergeCell ref="A16:A19"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A46:A53"/>
-    <mergeCell ref="B46:B53"/>
-    <mergeCell ref="A30:A34"/>
-    <mergeCell ref="B30:B34"/>
-    <mergeCell ref="A35:A45"/>
-    <mergeCell ref="B35:B45"/>
-    <mergeCell ref="A27:A29"/>
-    <mergeCell ref="B27:B29"/>
-    <mergeCell ref="B16:B21"/>
-    <mergeCell ref="B22:B26"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>